<commit_message>
Update 07-07-25: Añadido código para AVP y prevalencia para grupos quinquenales entre 35 y 80 años
</commit_message>
<xml_diff>
--- a/Bases de datos/clean/dic_arg_defun_avp.xlsx
+++ b/Bases de datos/clean/dic_arg_defun_avp.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -460,19 +460,19 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>20-24 años, 25-29 años, 30-34 años, 35-39 años, 40-44 años, 45-49 años, 50-54 años, 55-59 años, 60-64 años, 65-69 años, 70-74 años, 75-79 años, 80+ años</t>
+          <t>35-39, 40-44, 45-49, 50-54, 55-59, 60-64, 65-69, 70-74, 75-79, 80+</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>grupo_edad_10</t>
+          <t>sexo</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Grupo de edad decenal</t>
+          <t>Sexo biológico</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -482,41 +482,41 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>20-29 años, 30-39 años, 40-49 años, 50-59 años, 60-69 años, 70-79 años, 80+ años</t>
+          <t>Varón, Mujer</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>sexo</t>
+          <t>defun_n</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Sexo biológico</t>
+          <t>Número de defunciones para el trienio correspondiente</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>factor</t>
+          <t>numeric</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Varón, Mujer</t>
+          <t>0-Inf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>defun_n</t>
+          <t>defun_mean</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Número de defunciones para el trienio correspondiente</t>
+          <t>Promedio de defunciones para el trienio correspondiente</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -533,12 +533,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>defun_mean</t>
+          <t>lx</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Promedio de defunciones para el trienio correspondiente</t>
+          <t>Cantidad de personas vivas a la edad x</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -555,12 +555,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>lx</t>
+          <t>Tx</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Cantidad de personas vivas a la edad x</t>
+          <t>Años-persona vividos por encima de la edad x</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -577,12 +577,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Tx</t>
+          <t>ex</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Años-persona vividos por encima de la edad x</t>
+          <t>Esperanza de vida a la edad x</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -599,12 +599,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ex</t>
+          <t>AVP</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Esperanza de vida a la edad x</t>
+          <t>Años de vida perdidos por muerte prematura</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -613,28 +613,6 @@
         </is>
       </c>
       <c r="D12" t="inlineStr">
-        <is>
-          <t>0-Inf</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>AVP</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Años de vida perdidos por muerte prematura</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>numeric</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
         <is>
           <t>0-Inf</t>
         </is>

</xml_diff>

<commit_message>
Update 19-01-2026: Actualizado cálculo AVP
</commit_message>
<xml_diff>
--- a/Bases de datos/clean/dic_arg_defun_avp.xlsx
+++ b/Bases de datos/clean/dic_arg_defun_avp.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -372,7 +372,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>valor</t>
+          <t>niveles</t>
         </is>
       </c>
     </row>
@@ -384,7 +384,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Año de realización ENFR</t>
+          <t>Año de realización de la Encuesta Nacional de Factores de Riesgo (ENFR)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -401,12 +401,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>prov_id</t>
+          <t>codprov_censo</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Identificador numérico de provincia</t>
+          <t>Identificador numérico de provincia según clasificación INDEC</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -445,12 +445,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>grupo_edad_10</t>
+          <t>region_deis</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Grupo de edad decenal</t>
+          <t>Región geográfica según clasificación DEIS (2021)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -460,19 +460,19 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>30-39, 40-49, 50-59, 60-69, 70-79, 80+</t>
+          <t>Centro, Cuyo, NEA, NOA1, NOA2, Patagonia Norte, Patagonia Sur</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>sexo</t>
+          <t>grupo_edad_10</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Sexo biológico</t>
+          <t>Grupo de edad decenal</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -482,41 +482,41 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Varón, Mujer</t>
+          <t>30 a 39, 40 a 49, 50 a 59, 60 a 69, 70 a 79, 80+</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>defun_n</t>
+          <t>sexo</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Número de defunciones para el trienio correspondiente</t>
+          <t>Sexo biológico</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>numeric</t>
+          <t>factor</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>0-Inf</t>
+          <t>Mujer, Varón</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>defun_mean</t>
+          <t>defun_n</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Promedio de defunciones para el trienio correspondiente</t>
+          <t>Número de defunciones para el trienio correspondiente</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -526,19 +526,19 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0-Inf</t>
+          <t>O-Inf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>lx</t>
+          <t>defun_mean</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Cantidad de personas vivas a la edad x</t>
+          <t>Promedio de defunciones para el trienio correspondiente</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -548,19 +548,19 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0-Inf</t>
+          <t>O-Inf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Tx</t>
+          <t>lx</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Años-persona vividos por encima de la edad x</t>
+          <t>Cantidad de personas vivas a la edad x</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -570,19 +570,19 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0-Inf</t>
+          <t>O-Inf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ex</t>
+          <t>Tx</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Esperanza de vida a la edad x</t>
+          <t>Años-persona vividos por encima de la edad x</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -592,29 +592,51 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0-Inf</t>
+          <t>O-Inf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>ex</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Esperanza de vida a la edad x</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>O-Inf</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>AVP</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Años de vida perdidos por muerte prematura</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Años de vida perdidos por muerte prematura por diabetes mellitus</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
         <is>
           <t>numeric</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>0-Inf</t>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>O-Inf</t>
         </is>
       </c>
     </row>

</xml_diff>